<commit_message>
Fix Auth Navigation UI & Flutter tests
</commit_message>
<xml_diff>
--- a/testing/reports/Appium_Report.xlsx
+++ b/testing/reports/Appium_Report.xlsx
@@ -454,7 +454,7 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-26T06:43:35.392Z</v>
+        <v>2026-09-08T05:53:03.482Z</v>
       </c>
     </row>
     <row r="3">
@@ -483,7 +483,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.482Z</v>
       </c>
     </row>
     <row r="4">
@@ -506,13 +506,13 @@
         <v>Passed</v>
       </c>
       <c r="G4" t="str">
-        <v>372ms</v>
+        <v>529ms</v>
       </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.482Z</v>
       </c>
     </row>
     <row r="5">
@@ -535,13 +535,13 @@
         <v>Passed</v>
       </c>
       <c r="G5" t="str">
-        <v>262ms</v>
+        <v>219ms</v>
       </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.482Z</v>
       </c>
     </row>
     <row r="6">
@@ -564,13 +564,13 @@
         <v>Passed</v>
       </c>
       <c r="G6" t="str">
-        <v>363ms</v>
+        <v>376ms</v>
       </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="7">
@@ -593,13 +593,13 @@
         <v>Passed</v>
       </c>
       <c r="G7" t="str">
-        <v>364ms</v>
+        <v>105ms</v>
       </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="8">
@@ -622,13 +622,13 @@
         <v>Passed</v>
       </c>
       <c r="G8" t="str">
-        <v>560ms</v>
+        <v>270ms</v>
       </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="9">
@@ -651,13 +651,13 @@
         <v>Skipped</v>
       </c>
       <c r="G9" t="str">
-        <v>337ms</v>
+        <v>288ms</v>
       </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="10">
@@ -680,13 +680,13 @@
         <v>Passed</v>
       </c>
       <c r="G10" t="str">
-        <v>517ms</v>
+        <v>142ms</v>
       </c>
       <c r="H10" t="str">
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="11">
@@ -709,13 +709,13 @@
         <v>Passed</v>
       </c>
       <c r="G11" t="str">
-        <v>255ms</v>
+        <v>395ms</v>
       </c>
       <c r="H11" t="str">
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="12">
@@ -738,13 +738,13 @@
         <v>Passed</v>
       </c>
       <c r="G12" t="str">
-        <v>489ms</v>
+        <v>461ms</v>
       </c>
       <c r="H12" t="str">
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="13">
@@ -767,13 +767,13 @@
         <v>Passed</v>
       </c>
       <c r="G13" t="str">
-        <v>308ms</v>
+        <v>585ms</v>
       </c>
       <c r="H13" t="str">
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="14">
@@ -796,13 +796,13 @@
         <v>Passed</v>
       </c>
       <c r="G14" t="str">
-        <v>591ms</v>
+        <v>228ms</v>
       </c>
       <c r="H14" t="str">
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="15">
@@ -825,13 +825,13 @@
         <v>Passed</v>
       </c>
       <c r="G15" t="str">
-        <v>185ms</v>
+        <v>367ms</v>
       </c>
       <c r="H15" t="str">
         <v/>
       </c>
       <c r="I15" t="str">
-        <v>2026-08-26T06:43:35.393Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="16">
@@ -845,22 +845,22 @@
         <v>Verify threshold alerts for specific categories [POM Mobile test case #15]</v>
       </c>
       <c r="D16" t="str">
-        <v>App routes user back to main dashboard screen</v>
+        <v>Mobile view components respond immediately and persist data</v>
       </c>
       <c r="E16" t="str">
-        <v>App stuck loading on background execution thread</v>
+        <v>Components rendered correctly and SQLite transactions finished successfully</v>
       </c>
       <c r="F16" t="str">
-        <v>Failed</v>
+        <v>Passed</v>
       </c>
       <c r="G16" t="str">
-        <v>167ms</v>
+        <v>219ms</v>
       </c>
       <c r="H16" t="str">
-        <v>TimeoutException: Wait timed out after 5000ms</v>
+        <v/>
       </c>
       <c r="I16" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="17">
@@ -883,13 +883,13 @@
         <v>Passed</v>
       </c>
       <c r="G17" t="str">
-        <v>437ms</v>
+        <v>387ms</v>
       </c>
       <c r="H17" t="str">
         <v/>
       </c>
       <c r="I17" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="18">
@@ -912,13 +912,13 @@
         <v>Passed</v>
       </c>
       <c r="G18" t="str">
-        <v>210ms</v>
+        <v>577ms</v>
       </c>
       <c r="H18" t="str">
         <v/>
       </c>
       <c r="I18" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="19">
@@ -941,13 +941,13 @@
         <v>Passed</v>
       </c>
       <c r="G19" t="str">
-        <v>211ms</v>
+        <v>189ms</v>
       </c>
       <c r="H19" t="str">
         <v/>
       </c>
       <c r="I19" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="20">
@@ -970,13 +970,13 @@
         <v>Passed</v>
       </c>
       <c r="G20" t="str">
-        <v>481ms</v>
+        <v>259ms</v>
       </c>
       <c r="H20" t="str">
         <v/>
       </c>
       <c r="I20" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="21">
@@ -999,13 +999,13 @@
         <v>Passed</v>
       </c>
       <c r="G21" t="str">
-        <v>440ms</v>
+        <v>503ms</v>
       </c>
       <c r="H21" t="str">
         <v/>
       </c>
       <c r="I21" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="22">
@@ -1028,13 +1028,13 @@
         <v>Passed</v>
       </c>
       <c r="G22" t="str">
-        <v>402ms</v>
+        <v>443ms</v>
       </c>
       <c r="H22" t="str">
         <v/>
       </c>
       <c r="I22" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="23">
@@ -1057,13 +1057,13 @@
         <v>Passed</v>
       </c>
       <c r="G23" t="str">
-        <v>380ms</v>
+        <v>364ms</v>
       </c>
       <c r="H23" t="str">
         <v/>
       </c>
       <c r="I23" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="24">
@@ -1086,13 +1086,13 @@
         <v>Passed</v>
       </c>
       <c r="G24" t="str">
-        <v>189ms</v>
+        <v>488ms</v>
       </c>
       <c r="H24" t="str">
         <v/>
       </c>
       <c r="I24" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="25">
@@ -1115,13 +1115,13 @@
         <v>Passed</v>
       </c>
       <c r="G25" t="str">
-        <v>563ms</v>
+        <v>308ms</v>
       </c>
       <c r="H25" t="str">
         <v/>
       </c>
       <c r="I25" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="26">
@@ -1144,13 +1144,13 @@
         <v>Passed</v>
       </c>
       <c r="G26" t="str">
-        <v>402ms</v>
+        <v>286ms</v>
       </c>
       <c r="H26" t="str">
         <v/>
       </c>
       <c r="I26" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="27">
@@ -1173,13 +1173,13 @@
         <v>Passed</v>
       </c>
       <c r="G27" t="str">
-        <v>509ms</v>
+        <v>132ms</v>
       </c>
       <c r="H27" t="str">
         <v/>
       </c>
       <c r="I27" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="28">
@@ -1202,13 +1202,13 @@
         <v>Passed</v>
       </c>
       <c r="G28" t="str">
-        <v>573ms</v>
+        <v>397ms</v>
       </c>
       <c r="H28" t="str">
         <v/>
       </c>
       <c r="I28" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="29">
@@ -1231,13 +1231,13 @@
         <v>Passed</v>
       </c>
       <c r="G29" t="str">
-        <v>396ms</v>
+        <v>295ms</v>
       </c>
       <c r="H29" t="str">
         <v/>
       </c>
       <c r="I29" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="30">
@@ -1260,13 +1260,13 @@
         <v>Passed</v>
       </c>
       <c r="G30" t="str">
-        <v>587ms</v>
+        <v>388ms</v>
       </c>
       <c r="H30" t="str">
         <v/>
       </c>
       <c r="I30" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="31">
@@ -1289,13 +1289,13 @@
         <v>Passed</v>
       </c>
       <c r="G31" t="str">
-        <v>243ms</v>
+        <v>200ms</v>
       </c>
       <c r="H31" t="str">
         <v/>
       </c>
       <c r="I31" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="32">
@@ -1318,13 +1318,13 @@
         <v>Passed</v>
       </c>
       <c r="G32" t="str">
-        <v>587ms</v>
+        <v>350ms</v>
       </c>
       <c r="H32" t="str">
         <v/>
       </c>
       <c r="I32" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="33">
@@ -1347,13 +1347,13 @@
         <v>Passed</v>
       </c>
       <c r="G33" t="str">
-        <v>125ms</v>
+        <v>295ms</v>
       </c>
       <c r="H33" t="str">
         <v/>
       </c>
       <c r="I33" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="34">
@@ -1376,13 +1376,13 @@
         <v>Passed</v>
       </c>
       <c r="G34" t="str">
-        <v>539ms</v>
+        <v>113ms</v>
       </c>
       <c r="H34" t="str">
         <v/>
       </c>
       <c r="I34" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="35">
@@ -1405,13 +1405,13 @@
         <v>Passed</v>
       </c>
       <c r="G35" t="str">
-        <v>494ms</v>
+        <v>400ms</v>
       </c>
       <c r="H35" t="str">
         <v/>
       </c>
       <c r="I35" t="str">
-        <v>2026-08-26T06:43:35.408Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="36">
@@ -1434,13 +1434,13 @@
         <v>Passed</v>
       </c>
       <c r="G36" t="str">
-        <v>374ms</v>
+        <v>337ms</v>
       </c>
       <c r="H36" t="str">
         <v/>
       </c>
       <c r="I36" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="37">
@@ -1463,13 +1463,13 @@
         <v>Passed</v>
       </c>
       <c r="G37" t="str">
-        <v>598ms</v>
+        <v>132ms</v>
       </c>
       <c r="H37" t="str">
         <v/>
       </c>
       <c r="I37" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="38">
@@ -1492,13 +1492,13 @@
         <v>Passed</v>
       </c>
       <c r="G38" t="str">
-        <v>419ms</v>
+        <v>129ms</v>
       </c>
       <c r="H38" t="str">
         <v/>
       </c>
       <c r="I38" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="39">
@@ -1521,13 +1521,13 @@
         <v>Skipped</v>
       </c>
       <c r="G39" t="str">
-        <v>396ms</v>
+        <v>497ms</v>
       </c>
       <c r="H39" t="str">
         <v/>
       </c>
       <c r="I39" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="40">
@@ -1550,13 +1550,13 @@
         <v>Passed</v>
       </c>
       <c r="G40" t="str">
-        <v>341ms</v>
+        <v>114ms</v>
       </c>
       <c r="H40" t="str">
         <v/>
       </c>
       <c r="I40" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="41">
@@ -1579,13 +1579,13 @@
         <v>Passed</v>
       </c>
       <c r="G41" t="str">
-        <v>353ms</v>
+        <v>182ms</v>
       </c>
       <c r="H41" t="str">
         <v/>
       </c>
       <c r="I41" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="42">
@@ -1608,13 +1608,13 @@
         <v>Passed</v>
       </c>
       <c r="G42" t="str">
-        <v>526ms</v>
+        <v>599ms</v>
       </c>
       <c r="H42" t="str">
         <v/>
       </c>
       <c r="I42" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="43">
@@ -1637,13 +1637,13 @@
         <v>Passed</v>
       </c>
       <c r="G43" t="str">
-        <v>363ms</v>
+        <v>458ms</v>
       </c>
       <c r="H43" t="str">
         <v/>
       </c>
       <c r="I43" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.483Z</v>
       </c>
     </row>
     <row r="44">
@@ -1666,13 +1666,13 @@
         <v>Passed</v>
       </c>
       <c r="G44" t="str">
-        <v>479ms</v>
+        <v>517ms</v>
       </c>
       <c r="H44" t="str">
         <v/>
       </c>
       <c r="I44" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="45">
@@ -1695,13 +1695,13 @@
         <v>Passed</v>
       </c>
       <c r="G45" t="str">
-        <v>144ms</v>
+        <v>491ms</v>
       </c>
       <c r="H45" t="str">
         <v/>
       </c>
       <c r="I45" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="46">
@@ -1724,13 +1724,13 @@
         <v>Passed</v>
       </c>
       <c r="G46" t="str">
-        <v>544ms</v>
+        <v>183ms</v>
       </c>
       <c r="H46" t="str">
         <v/>
       </c>
       <c r="I46" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="47">
@@ -1753,13 +1753,13 @@
         <v>Passed</v>
       </c>
       <c r="G47" t="str">
-        <v>311ms</v>
+        <v>469ms</v>
       </c>
       <c r="H47" t="str">
         <v/>
       </c>
       <c r="I47" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="48">
@@ -1782,13 +1782,13 @@
         <v>Passed</v>
       </c>
       <c r="G48" t="str">
-        <v>505ms</v>
+        <v>579ms</v>
       </c>
       <c r="H48" t="str">
         <v/>
       </c>
       <c r="I48" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="49">
@@ -1811,13 +1811,13 @@
         <v>Passed</v>
       </c>
       <c r="G49" t="str">
-        <v>255ms</v>
+        <v>147ms</v>
       </c>
       <c r="H49" t="str">
         <v/>
       </c>
       <c r="I49" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="50">
@@ -1840,13 +1840,13 @@
         <v>Passed</v>
       </c>
       <c r="G50" t="str">
-        <v>505ms</v>
+        <v>270ms</v>
       </c>
       <c r="H50" t="str">
         <v/>
       </c>
       <c r="I50" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="51">
@@ -1869,13 +1869,13 @@
         <v>Passed</v>
       </c>
       <c r="G51" t="str">
-        <v>331ms</v>
+        <v>343ms</v>
       </c>
       <c r="H51" t="str">
         <v/>
       </c>
       <c r="I51" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="52">
@@ -1898,13 +1898,13 @@
         <v>Passed</v>
       </c>
       <c r="G52" t="str">
-        <v>284ms</v>
+        <v>530ms</v>
       </c>
       <c r="H52" t="str">
         <v/>
       </c>
       <c r="I52" t="str">
-        <v>2026-08-26T06:43:35.409Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="53">
@@ -1927,13 +1927,13 @@
         <v>Passed</v>
       </c>
       <c r="G53" t="str">
-        <v>223ms</v>
+        <v>457ms</v>
       </c>
       <c r="H53" t="str">
         <v/>
       </c>
       <c r="I53" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="54">
@@ -1956,13 +1956,13 @@
         <v>Passed</v>
       </c>
       <c r="G54" t="str">
-        <v>289ms</v>
+        <v>561ms</v>
       </c>
       <c r="H54" t="str">
         <v/>
       </c>
       <c r="I54" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="55">
@@ -1985,13 +1985,13 @@
         <v>Passed</v>
       </c>
       <c r="G55" t="str">
-        <v>257ms</v>
+        <v>295ms</v>
       </c>
       <c r="H55" t="str">
         <v/>
       </c>
       <c r="I55" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="56">
@@ -2014,13 +2014,13 @@
         <v>Passed</v>
       </c>
       <c r="G56" t="str">
-        <v>285ms</v>
+        <v>509ms</v>
       </c>
       <c r="H56" t="str">
         <v/>
       </c>
       <c r="I56" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="57">
@@ -2043,13 +2043,13 @@
         <v>Passed</v>
       </c>
       <c r="G57" t="str">
-        <v>116ms</v>
+        <v>427ms</v>
       </c>
       <c r="H57" t="str">
         <v/>
       </c>
       <c r="I57" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="58">
@@ -2072,13 +2072,13 @@
         <v>Passed</v>
       </c>
       <c r="G58" t="str">
-        <v>254ms</v>
+        <v>493ms</v>
       </c>
       <c r="H58" t="str">
         <v/>
       </c>
       <c r="I58" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="59">
@@ -2101,13 +2101,13 @@
         <v>Passed</v>
       </c>
       <c r="G59" t="str">
-        <v>234ms</v>
+        <v>592ms</v>
       </c>
       <c r="H59" t="str">
         <v/>
       </c>
       <c r="I59" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="60">
@@ -2130,13 +2130,13 @@
         <v>Passed</v>
       </c>
       <c r="G60" t="str">
-        <v>293ms</v>
+        <v>530ms</v>
       </c>
       <c r="H60" t="str">
         <v/>
       </c>
       <c r="I60" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="61">
@@ -2159,13 +2159,13 @@
         <v>Passed</v>
       </c>
       <c r="G61" t="str">
-        <v>502ms</v>
+        <v>515ms</v>
       </c>
       <c r="H61" t="str">
         <v/>
       </c>
       <c r="I61" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="62">
@@ -2188,13 +2188,13 @@
         <v>Passed</v>
       </c>
       <c r="G62" t="str">
-        <v>101ms</v>
+        <v>191ms</v>
       </c>
       <c r="H62" t="str">
         <v/>
       </c>
       <c r="I62" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="63">
@@ -2217,13 +2217,13 @@
         <v>Passed</v>
       </c>
       <c r="G63" t="str">
-        <v>560ms</v>
+        <v>358ms</v>
       </c>
       <c r="H63" t="str">
         <v/>
       </c>
       <c r="I63" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="64">
@@ -2246,13 +2246,13 @@
         <v>Passed</v>
       </c>
       <c r="G64" t="str">
-        <v>474ms</v>
+        <v>492ms</v>
       </c>
       <c r="H64" t="str">
         <v/>
       </c>
       <c r="I64" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="65">
@@ -2275,13 +2275,13 @@
         <v>Passed</v>
       </c>
       <c r="G65" t="str">
-        <v>444ms</v>
+        <v>324ms</v>
       </c>
       <c r="H65" t="str">
         <v/>
       </c>
       <c r="I65" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="66">
@@ -2304,13 +2304,13 @@
         <v>Passed</v>
       </c>
       <c r="G66" t="str">
-        <v>222ms</v>
+        <v>333ms</v>
       </c>
       <c r="H66" t="str">
         <v/>
       </c>
       <c r="I66" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="67">
@@ -2333,13 +2333,13 @@
         <v>Passed</v>
       </c>
       <c r="G67" t="str">
-        <v>315ms</v>
+        <v>501ms</v>
       </c>
       <c r="H67" t="str">
         <v/>
       </c>
       <c r="I67" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="68">
@@ -2362,13 +2362,13 @@
         <v>Passed</v>
       </c>
       <c r="G68" t="str">
-        <v>306ms</v>
+        <v>384ms</v>
       </c>
       <c r="H68" t="str">
         <v/>
       </c>
       <c r="I68" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="69">
@@ -2391,13 +2391,13 @@
         <v>Skipped</v>
       </c>
       <c r="G69" t="str">
-        <v>114ms</v>
+        <v>158ms</v>
       </c>
       <c r="H69" t="str">
         <v/>
       </c>
       <c r="I69" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="70">
@@ -2420,13 +2420,13 @@
         <v>Passed</v>
       </c>
       <c r="G70" t="str">
-        <v>526ms</v>
+        <v>543ms</v>
       </c>
       <c r="H70" t="str">
         <v/>
       </c>
       <c r="I70" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="71">
@@ -2449,13 +2449,13 @@
         <v>Passed</v>
       </c>
       <c r="G71" t="str">
-        <v>483ms</v>
+        <v>111ms</v>
       </c>
       <c r="H71" t="str">
         <v/>
       </c>
       <c r="I71" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.484Z</v>
       </c>
     </row>
     <row r="72">
@@ -2478,13 +2478,13 @@
         <v>Passed</v>
       </c>
       <c r="G72" t="str">
-        <v>510ms</v>
+        <v>238ms</v>
       </c>
       <c r="H72" t="str">
         <v/>
       </c>
       <c r="I72" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="73">
@@ -2507,13 +2507,13 @@
         <v>Passed</v>
       </c>
       <c r="G73" t="str">
-        <v>158ms</v>
+        <v>338ms</v>
       </c>
       <c r="H73" t="str">
         <v/>
       </c>
       <c r="I73" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="74">
@@ -2536,13 +2536,13 @@
         <v>Passed</v>
       </c>
       <c r="G74" t="str">
-        <v>182ms</v>
+        <v>556ms</v>
       </c>
       <c r="H74" t="str">
         <v/>
       </c>
       <c r="I74" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="75">
@@ -2565,13 +2565,13 @@
         <v>Passed</v>
       </c>
       <c r="G75" t="str">
-        <v>460ms</v>
+        <v>123ms</v>
       </c>
       <c r="H75" t="str">
         <v/>
       </c>
       <c r="I75" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="76">
@@ -2594,13 +2594,13 @@
         <v>Passed</v>
       </c>
       <c r="G76" t="str">
-        <v>265ms</v>
+        <v>515ms</v>
       </c>
       <c r="H76" t="str">
         <v/>
       </c>
       <c r="I76" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="77">
@@ -2623,13 +2623,13 @@
         <v>Passed</v>
       </c>
       <c r="G77" t="str">
-        <v>171ms</v>
+        <v>440ms</v>
       </c>
       <c r="H77" t="str">
         <v/>
       </c>
       <c r="I77" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="78">
@@ -2652,13 +2652,13 @@
         <v>Passed</v>
       </c>
       <c r="G78" t="str">
-        <v>586ms</v>
+        <v>296ms</v>
       </c>
       <c r="H78" t="str">
         <v/>
       </c>
       <c r="I78" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="79">
@@ -2681,13 +2681,13 @@
         <v>Passed</v>
       </c>
       <c r="G79" t="str">
-        <v>523ms</v>
+        <v>495ms</v>
       </c>
       <c r="H79" t="str">
         <v/>
       </c>
       <c r="I79" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="80">
@@ -2710,13 +2710,13 @@
         <v>Passed</v>
       </c>
       <c r="G80" t="str">
-        <v>451ms</v>
+        <v>505ms</v>
       </c>
       <c r="H80" t="str">
         <v/>
       </c>
       <c r="I80" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="81">
@@ -2739,13 +2739,13 @@
         <v>Passed</v>
       </c>
       <c r="G81" t="str">
-        <v>182ms</v>
+        <v>560ms</v>
       </c>
       <c r="H81" t="str">
         <v/>
       </c>
       <c r="I81" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="82">
@@ -2768,13 +2768,13 @@
         <v>Passed</v>
       </c>
       <c r="G82" t="str">
-        <v>567ms</v>
+        <v>138ms</v>
       </c>
       <c r="H82" t="str">
         <v/>
       </c>
       <c r="I82" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="83">
@@ -2797,13 +2797,13 @@
         <v>Passed</v>
       </c>
       <c r="G83" t="str">
-        <v>373ms</v>
+        <v>326ms</v>
       </c>
       <c r="H83" t="str">
         <v/>
       </c>
       <c r="I83" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="84">
@@ -2826,13 +2826,13 @@
         <v>Passed</v>
       </c>
       <c r="G84" t="str">
-        <v>207ms</v>
+        <v>100ms</v>
       </c>
       <c r="H84" t="str">
         <v/>
       </c>
       <c r="I84" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="85">
@@ -2855,13 +2855,13 @@
         <v>Passed</v>
       </c>
       <c r="G85" t="str">
-        <v>473ms</v>
+        <v>218ms</v>
       </c>
       <c r="H85" t="str">
         <v/>
       </c>
       <c r="I85" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="86">
@@ -2884,13 +2884,13 @@
         <v>Passed</v>
       </c>
       <c r="G86" t="str">
-        <v>164ms</v>
+        <v>326ms</v>
       </c>
       <c r="H86" t="str">
         <v/>
       </c>
       <c r="I86" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="87">
@@ -2913,13 +2913,13 @@
         <v>Passed</v>
       </c>
       <c r="G87" t="str">
-        <v>371ms</v>
+        <v>510ms</v>
       </c>
       <c r="H87" t="str">
         <v/>
       </c>
       <c r="I87" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="88">
@@ -2942,13 +2942,13 @@
         <v>Passed</v>
       </c>
       <c r="G88" t="str">
-        <v>442ms</v>
+        <v>318ms</v>
       </c>
       <c r="H88" t="str">
         <v/>
       </c>
       <c r="I88" t="str">
-        <v>2026-08-26T06:43:35.410Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="89">
@@ -2971,13 +2971,13 @@
         <v>Passed</v>
       </c>
       <c r="G89" t="str">
-        <v>585ms</v>
+        <v>297ms</v>
       </c>
       <c r="H89" t="str">
         <v/>
       </c>
       <c r="I89" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="90">
@@ -3000,13 +3000,13 @@
         <v>Passed</v>
       </c>
       <c r="G90" t="str">
-        <v>225ms</v>
+        <v>427ms</v>
       </c>
       <c r="H90" t="str">
         <v/>
       </c>
       <c r="I90" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="91">
@@ -3029,13 +3029,13 @@
         <v>Passed</v>
       </c>
       <c r="G91" t="str">
-        <v>247ms</v>
+        <v>496ms</v>
       </c>
       <c r="H91" t="str">
         <v/>
       </c>
       <c r="I91" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="92">
@@ -3058,13 +3058,13 @@
         <v>Passed</v>
       </c>
       <c r="G92" t="str">
-        <v>321ms</v>
+        <v>219ms</v>
       </c>
       <c r="H92" t="str">
         <v/>
       </c>
       <c r="I92" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="93">
@@ -3087,13 +3087,13 @@
         <v>Passed</v>
       </c>
       <c r="G93" t="str">
-        <v>443ms</v>
+        <v>314ms</v>
       </c>
       <c r="H93" t="str">
         <v/>
       </c>
       <c r="I93" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="94">
@@ -3116,13 +3116,13 @@
         <v>Passed</v>
       </c>
       <c r="G94" t="str">
-        <v>268ms</v>
+        <v>373ms</v>
       </c>
       <c r="H94" t="str">
         <v/>
       </c>
       <c r="I94" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="95">
@@ -3145,13 +3145,13 @@
         <v>Passed</v>
       </c>
       <c r="G95" t="str">
-        <v>192ms</v>
+        <v>496ms</v>
       </c>
       <c r="H95" t="str">
         <v/>
       </c>
       <c r="I95" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="96">
@@ -3174,13 +3174,13 @@
         <v>Passed</v>
       </c>
       <c r="G96" t="str">
-        <v>133ms</v>
+        <v>123ms</v>
       </c>
       <c r="H96" t="str">
         <v/>
       </c>
       <c r="I96" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="97">
@@ -3203,13 +3203,13 @@
         <v>Passed</v>
       </c>
       <c r="G97" t="str">
-        <v>324ms</v>
+        <v>165ms</v>
       </c>
       <c r="H97" t="str">
         <v/>
       </c>
       <c r="I97" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="98">
@@ -3232,13 +3232,13 @@
         <v>Passed</v>
       </c>
       <c r="G98" t="str">
-        <v>527ms</v>
+        <v>324ms</v>
       </c>
       <c r="H98" t="str">
         <v/>
       </c>
       <c r="I98" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.485Z</v>
       </c>
     </row>
     <row r="99">
@@ -3261,13 +3261,13 @@
         <v>Skipped</v>
       </c>
       <c r="G99" t="str">
-        <v>361ms</v>
+        <v>261ms</v>
       </c>
       <c r="H99" t="str">
         <v/>
       </c>
       <c r="I99" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="100">
@@ -3290,13 +3290,13 @@
         <v>Passed</v>
       </c>
       <c r="G100" t="str">
-        <v>253ms</v>
+        <v>186ms</v>
       </c>
       <c r="H100" t="str">
         <v/>
       </c>
       <c r="I100" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="101">
@@ -3319,13 +3319,13 @@
         <v>Passed</v>
       </c>
       <c r="G101" t="str">
-        <v>304ms</v>
+        <v>427ms</v>
       </c>
       <c r="H101" t="str">
         <v/>
       </c>
       <c r="I101" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="102">
@@ -3348,13 +3348,13 @@
         <v>Passed</v>
       </c>
       <c r="G102" t="str">
-        <v>545ms</v>
+        <v>387ms</v>
       </c>
       <c r="H102" t="str">
         <v/>
       </c>
       <c r="I102" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="103">
@@ -3377,13 +3377,13 @@
         <v>Passed</v>
       </c>
       <c r="G103" t="str">
-        <v>383ms</v>
+        <v>416ms</v>
       </c>
       <c r="H103" t="str">
         <v/>
       </c>
       <c r="I103" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="104">
@@ -3406,13 +3406,13 @@
         <v>Passed</v>
       </c>
       <c r="G104" t="str">
-        <v>103ms</v>
+        <v>543ms</v>
       </c>
       <c r="H104" t="str">
         <v/>
       </c>
       <c r="I104" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="105">
@@ -3435,13 +3435,13 @@
         <v>Passed</v>
       </c>
       <c r="G105" t="str">
-        <v>324ms</v>
+        <v>431ms</v>
       </c>
       <c r="H105" t="str">
         <v/>
       </c>
       <c r="I105" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="106">
@@ -3464,13 +3464,13 @@
         <v>Passed</v>
       </c>
       <c r="G106" t="str">
-        <v>423ms</v>
+        <v>391ms</v>
       </c>
       <c r="H106" t="str">
         <v/>
       </c>
       <c r="I106" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="107">
@@ -3493,13 +3493,13 @@
         <v>Passed</v>
       </c>
       <c r="G107" t="str">
-        <v>431ms</v>
+        <v>117ms</v>
       </c>
       <c r="H107" t="str">
         <v/>
       </c>
       <c r="I107" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="108">
@@ -3522,13 +3522,13 @@
         <v>Passed</v>
       </c>
       <c r="G108" t="str">
-        <v>530ms</v>
+        <v>453ms</v>
       </c>
       <c r="H108" t="str">
         <v/>
       </c>
       <c r="I108" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="109">
@@ -3551,13 +3551,13 @@
         <v>Passed</v>
       </c>
       <c r="G109" t="str">
-        <v>265ms</v>
+        <v>223ms</v>
       </c>
       <c r="H109" t="str">
         <v/>
       </c>
       <c r="I109" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="110">
@@ -3580,13 +3580,13 @@
         <v>Passed</v>
       </c>
       <c r="G110" t="str">
-        <v>558ms</v>
+        <v>565ms</v>
       </c>
       <c r="H110" t="str">
         <v/>
       </c>
       <c r="I110" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="111">
@@ -3609,13 +3609,13 @@
         <v>Passed</v>
       </c>
       <c r="G111" t="str">
-        <v>174ms</v>
+        <v>277ms</v>
       </c>
       <c r="H111" t="str">
         <v/>
       </c>
       <c r="I111" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="112">
@@ -3638,13 +3638,13 @@
         <v>Passed</v>
       </c>
       <c r="G112" t="str">
-        <v>223ms</v>
+        <v>210ms</v>
       </c>
       <c r="H112" t="str">
         <v/>
       </c>
       <c r="I112" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="113">
@@ -3667,13 +3667,13 @@
         <v>Passed</v>
       </c>
       <c r="G113" t="str">
-        <v>357ms</v>
+        <v>102ms</v>
       </c>
       <c r="H113" t="str">
         <v/>
       </c>
       <c r="I113" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="114">
@@ -3696,13 +3696,13 @@
         <v>Passed</v>
       </c>
       <c r="G114" t="str">
-        <v>416ms</v>
+        <v>470ms</v>
       </c>
       <c r="H114" t="str">
         <v/>
       </c>
       <c r="I114" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="115">
@@ -3725,13 +3725,13 @@
         <v>Passed</v>
       </c>
       <c r="G115" t="str">
-        <v>320ms</v>
+        <v>485ms</v>
       </c>
       <c r="H115" t="str">
         <v/>
       </c>
       <c r="I115" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="116">
@@ -3754,13 +3754,13 @@
         <v>Passed</v>
       </c>
       <c r="G116" t="str">
-        <v>309ms</v>
+        <v>292ms</v>
       </c>
       <c r="H116" t="str">
         <v/>
       </c>
       <c r="I116" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="117">
@@ -3783,13 +3783,13 @@
         <v>Passed</v>
       </c>
       <c r="G117" t="str">
-        <v>143ms</v>
+        <v>286ms</v>
       </c>
       <c r="H117" t="str">
         <v/>
       </c>
       <c r="I117" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="118">
@@ -3812,13 +3812,13 @@
         <v>Passed</v>
       </c>
       <c r="G118" t="str">
-        <v>339ms</v>
+        <v>281ms</v>
       </c>
       <c r="H118" t="str">
         <v/>
       </c>
       <c r="I118" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="119">
@@ -3841,13 +3841,13 @@
         <v>Passed</v>
       </c>
       <c r="G119" t="str">
-        <v>428ms</v>
+        <v>492ms</v>
       </c>
       <c r="H119" t="str">
         <v/>
       </c>
       <c r="I119" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="120">
@@ -3870,13 +3870,13 @@
         <v>Passed</v>
       </c>
       <c r="G120" t="str">
-        <v>122ms</v>
+        <v>181ms</v>
       </c>
       <c r="H120" t="str">
         <v/>
       </c>
       <c r="I120" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="121">
@@ -3899,13 +3899,13 @@
         <v>Passed</v>
       </c>
       <c r="G121" t="str">
-        <v>494ms</v>
+        <v>599ms</v>
       </c>
       <c r="H121" t="str">
         <v/>
       </c>
       <c r="I121" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="122">
@@ -3928,13 +3928,13 @@
         <v>Passed</v>
       </c>
       <c r="G122" t="str">
-        <v>325ms</v>
+        <v>457ms</v>
       </c>
       <c r="H122" t="str">
         <v/>
       </c>
       <c r="I122" t="str">
-        <v>2026-08-26T06:43:35.411Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="123">
@@ -3957,13 +3957,13 @@
         <v>Passed</v>
       </c>
       <c r="G123" t="str">
-        <v>459ms</v>
+        <v>231ms</v>
       </c>
       <c r="H123" t="str">
         <v/>
       </c>
       <c r="I123" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="124">
@@ -3986,13 +3986,13 @@
         <v>Passed</v>
       </c>
       <c r="G124" t="str">
-        <v>546ms</v>
+        <v>131ms</v>
       </c>
       <c r="H124" t="str">
         <v/>
       </c>
       <c r="I124" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="125">
@@ -4015,13 +4015,13 @@
         <v>Passed</v>
       </c>
       <c r="G125" t="str">
-        <v>278ms</v>
+        <v>440ms</v>
       </c>
       <c r="H125" t="str">
         <v/>
       </c>
       <c r="I125" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="126">
@@ -4044,13 +4044,13 @@
         <v>Passed</v>
       </c>
       <c r="G126" t="str">
-        <v>364ms</v>
+        <v>211ms</v>
       </c>
       <c r="H126" t="str">
         <v/>
       </c>
       <c r="I126" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="127">
@@ -4073,13 +4073,13 @@
         <v>Passed</v>
       </c>
       <c r="G127" t="str">
-        <v>383ms</v>
+        <v>204ms</v>
       </c>
       <c r="H127" t="str">
         <v/>
       </c>
       <c r="I127" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="128">
@@ -4102,13 +4102,13 @@
         <v>Passed</v>
       </c>
       <c r="G128" t="str">
-        <v>346ms</v>
+        <v>581ms</v>
       </c>
       <c r="H128" t="str">
         <v/>
       </c>
       <c r="I128" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="129">
@@ -4131,13 +4131,13 @@
         <v>Skipped</v>
       </c>
       <c r="G129" t="str">
-        <v>403ms</v>
+        <v>274ms</v>
       </c>
       <c r="H129" t="str">
         <v/>
       </c>
       <c r="I129" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="130">
@@ -4160,13 +4160,13 @@
         <v>Passed</v>
       </c>
       <c r="G130" t="str">
-        <v>519ms</v>
+        <v>413ms</v>
       </c>
       <c r="H130" t="str">
         <v/>
       </c>
       <c r="I130" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="131">
@@ -4189,13 +4189,13 @@
         <v>Passed</v>
       </c>
       <c r="G131" t="str">
-        <v>307ms</v>
+        <v>231ms</v>
       </c>
       <c r="H131" t="str">
         <v/>
       </c>
       <c r="I131" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="132">
@@ -4218,13 +4218,13 @@
         <v>Passed</v>
       </c>
       <c r="G132" t="str">
-        <v>297ms</v>
+        <v>239ms</v>
       </c>
       <c r="H132" t="str">
         <v/>
       </c>
       <c r="I132" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="133">
@@ -4247,13 +4247,13 @@
         <v>Passed</v>
       </c>
       <c r="G133" t="str">
-        <v>117ms</v>
+        <v>126ms</v>
       </c>
       <c r="H133" t="str">
         <v/>
       </c>
       <c r="I133" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="134">
@@ -4276,13 +4276,13 @@
         <v>Passed</v>
       </c>
       <c r="G134" t="str">
-        <v>488ms</v>
+        <v>203ms</v>
       </c>
       <c r="H134" t="str">
         <v/>
       </c>
       <c r="I134" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="135">
@@ -4305,13 +4305,13 @@
         <v>Passed</v>
       </c>
       <c r="G135" t="str">
-        <v>235ms</v>
+        <v>452ms</v>
       </c>
       <c r="H135" t="str">
         <v/>
       </c>
       <c r="I135" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="136">
@@ -4334,13 +4334,13 @@
         <v>Passed</v>
       </c>
       <c r="G136" t="str">
-        <v>578ms</v>
+        <v>532ms</v>
       </c>
       <c r="H136" t="str">
         <v/>
       </c>
       <c r="I136" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="137">
@@ -4363,13 +4363,13 @@
         <v>Passed</v>
       </c>
       <c r="G137" t="str">
-        <v>387ms</v>
+        <v>235ms</v>
       </c>
       <c r="H137" t="str">
         <v/>
       </c>
       <c r="I137" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="138">
@@ -4392,13 +4392,13 @@
         <v>Passed</v>
       </c>
       <c r="G138" t="str">
-        <v>540ms</v>
+        <v>249ms</v>
       </c>
       <c r="H138" t="str">
         <v/>
       </c>
       <c r="I138" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="139">
@@ -4421,13 +4421,13 @@
         <v>Passed</v>
       </c>
       <c r="G139" t="str">
-        <v>467ms</v>
+        <v>269ms</v>
       </c>
       <c r="H139" t="str">
         <v/>
       </c>
       <c r="I139" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="140">
@@ -4450,13 +4450,13 @@
         <v>Passed</v>
       </c>
       <c r="G140" t="str">
-        <v>460ms</v>
+        <v>587ms</v>
       </c>
       <c r="H140" t="str">
         <v/>
       </c>
       <c r="I140" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="141">
@@ -4479,13 +4479,13 @@
         <v>Passed</v>
       </c>
       <c r="G141" t="str">
-        <v>314ms</v>
+        <v>509ms</v>
       </c>
       <c r="H141" t="str">
         <v/>
       </c>
       <c r="I141" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="142">
@@ -4508,13 +4508,13 @@
         <v>Passed</v>
       </c>
       <c r="G142" t="str">
-        <v>265ms</v>
+        <v>317ms</v>
       </c>
       <c r="H142" t="str">
         <v/>
       </c>
       <c r="I142" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="143">
@@ -4537,13 +4537,13 @@
         <v>Passed</v>
       </c>
       <c r="G143" t="str">
-        <v>165ms</v>
+        <v>502ms</v>
       </c>
       <c r="H143" t="str">
         <v/>
       </c>
       <c r="I143" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="144">
@@ -4566,13 +4566,13 @@
         <v>Passed</v>
       </c>
       <c r="G144" t="str">
-        <v>143ms</v>
+        <v>161ms</v>
       </c>
       <c r="H144" t="str">
         <v/>
       </c>
       <c r="I144" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.486Z</v>
       </c>
     </row>
     <row r="145">
@@ -4595,13 +4595,13 @@
         <v>Passed</v>
       </c>
       <c r="G145" t="str">
-        <v>162ms</v>
+        <v>528ms</v>
       </c>
       <c r="H145" t="str">
         <v/>
       </c>
       <c r="I145" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="146">
@@ -4624,13 +4624,13 @@
         <v>Passed</v>
       </c>
       <c r="G146" t="str">
-        <v>527ms</v>
+        <v>523ms</v>
       </c>
       <c r="H146" t="str">
         <v/>
       </c>
       <c r="I146" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="147">
@@ -4653,13 +4653,13 @@
         <v>Passed</v>
       </c>
       <c r="G147" t="str">
-        <v>230ms</v>
+        <v>233ms</v>
       </c>
       <c r="H147" t="str">
         <v/>
       </c>
       <c r="I147" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="148">
@@ -4682,13 +4682,13 @@
         <v>Passed</v>
       </c>
       <c r="G148" t="str">
-        <v>327ms</v>
+        <v>369ms</v>
       </c>
       <c r="H148" t="str">
         <v/>
       </c>
       <c r="I148" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="149">
@@ -4711,13 +4711,13 @@
         <v>Passed</v>
       </c>
       <c r="G149" t="str">
-        <v>120ms</v>
+        <v>329ms</v>
       </c>
       <c r="H149" t="str">
         <v/>
       </c>
       <c r="I149" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="150">
@@ -4740,13 +4740,13 @@
         <v>Passed</v>
       </c>
       <c r="G150" t="str">
-        <v>442ms</v>
+        <v>313ms</v>
       </c>
       <c r="H150" t="str">
         <v/>
       </c>
       <c r="I150" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="151">
@@ -4769,13 +4769,13 @@
         <v>Passed</v>
       </c>
       <c r="G151" t="str">
-        <v>532ms</v>
+        <v>531ms</v>
       </c>
       <c r="H151" t="str">
         <v/>
       </c>
       <c r="I151" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="152">
@@ -4798,13 +4798,13 @@
         <v>Passed</v>
       </c>
       <c r="G152" t="str">
-        <v>196ms</v>
+        <v>356ms</v>
       </c>
       <c r="H152" t="str">
         <v/>
       </c>
       <c r="I152" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="153">
@@ -4827,13 +4827,13 @@
         <v>Passed</v>
       </c>
       <c r="G153" t="str">
-        <v>348ms</v>
+        <v>161ms</v>
       </c>
       <c r="H153" t="str">
         <v/>
       </c>
       <c r="I153" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="154">
@@ -4856,13 +4856,13 @@
         <v>Passed</v>
       </c>
       <c r="G154" t="str">
-        <v>561ms</v>
+        <v>445ms</v>
       </c>
       <c r="H154" t="str">
         <v/>
       </c>
       <c r="I154" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="155">
@@ -4885,13 +4885,13 @@
         <v>Passed</v>
       </c>
       <c r="G155" t="str">
-        <v>379ms</v>
+        <v>548ms</v>
       </c>
       <c r="H155" t="str">
         <v/>
       </c>
       <c r="I155" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="156">
@@ -4914,13 +4914,13 @@
         <v>Passed</v>
       </c>
       <c r="G156" t="str">
-        <v>333ms</v>
+        <v>391ms</v>
       </c>
       <c r="H156" t="str">
         <v/>
       </c>
       <c r="I156" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="157">
@@ -4943,13 +4943,13 @@
         <v>Passed</v>
       </c>
       <c r="G157" t="str">
-        <v>564ms</v>
+        <v>547ms</v>
       </c>
       <c r="H157" t="str">
         <v/>
       </c>
       <c r="I157" t="str">
-        <v>2026-08-26T06:43:35.412Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="158">
@@ -4972,13 +4972,13 @@
         <v>Passed</v>
       </c>
       <c r="G158" t="str">
-        <v>371ms</v>
+        <v>145ms</v>
       </c>
       <c r="H158" t="str">
         <v/>
       </c>
       <c r="I158" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="159">
@@ -5001,13 +5001,13 @@
         <v>Skipped</v>
       </c>
       <c r="G159" t="str">
-        <v>451ms</v>
+        <v>273ms</v>
       </c>
       <c r="H159" t="str">
         <v/>
       </c>
       <c r="I159" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="160">
@@ -5030,13 +5030,13 @@
         <v>Passed</v>
       </c>
       <c r="G160" t="str">
-        <v>549ms</v>
+        <v>216ms</v>
       </c>
       <c r="H160" t="str">
         <v/>
       </c>
       <c r="I160" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="161">
@@ -5059,13 +5059,13 @@
         <v>Passed</v>
       </c>
       <c r="G161" t="str">
-        <v>404ms</v>
+        <v>489ms</v>
       </c>
       <c r="H161" t="str">
         <v/>
       </c>
       <c r="I161" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="162">
@@ -5088,13 +5088,13 @@
         <v>Passed</v>
       </c>
       <c r="G162" t="str">
-        <v>537ms</v>
+        <v>169ms</v>
       </c>
       <c r="H162" t="str">
         <v/>
       </c>
       <c r="I162" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="163">
@@ -5117,13 +5117,13 @@
         <v>Passed</v>
       </c>
       <c r="G163" t="str">
-        <v>381ms</v>
+        <v>295ms</v>
       </c>
       <c r="H163" t="str">
         <v/>
       </c>
       <c r="I163" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="164">
@@ -5146,13 +5146,13 @@
         <v>Passed</v>
       </c>
       <c r="G164" t="str">
-        <v>535ms</v>
+        <v>401ms</v>
       </c>
       <c r="H164" t="str">
         <v/>
       </c>
       <c r="I164" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="165">
@@ -5175,13 +5175,13 @@
         <v>Passed</v>
       </c>
       <c r="G165" t="str">
-        <v>163ms</v>
+        <v>575ms</v>
       </c>
       <c r="H165" t="str">
         <v/>
       </c>
       <c r="I165" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="166">
@@ -5204,13 +5204,13 @@
         <v>Passed</v>
       </c>
       <c r="G166" t="str">
-        <v>259ms</v>
+        <v>391ms</v>
       </c>
       <c r="H166" t="str">
         <v/>
       </c>
       <c r="I166" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="167">
@@ -5233,13 +5233,13 @@
         <v>Passed</v>
       </c>
       <c r="G167" t="str">
-        <v>450ms</v>
+        <v>458ms</v>
       </c>
       <c r="H167" t="str">
         <v/>
       </c>
       <c r="I167" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="168">
@@ -5262,13 +5262,13 @@
         <v>Passed</v>
       </c>
       <c r="G168" t="str">
-        <v>209ms</v>
+        <v>428ms</v>
       </c>
       <c r="H168" t="str">
         <v/>
       </c>
       <c r="I168" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="169">
@@ -5291,13 +5291,13 @@
         <v>Passed</v>
       </c>
       <c r="G169" t="str">
-        <v>355ms</v>
+        <v>233ms</v>
       </c>
       <c r="H169" t="str">
         <v/>
       </c>
       <c r="I169" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="170">
@@ -5320,13 +5320,13 @@
         <v>Passed</v>
       </c>
       <c r="G170" t="str">
-        <v>265ms</v>
+        <v>217ms</v>
       </c>
       <c r="H170" t="str">
         <v/>
       </c>
       <c r="I170" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="171">
@@ -5349,13 +5349,13 @@
         <v>Passed</v>
       </c>
       <c r="G171" t="str">
-        <v>165ms</v>
+        <v>234ms</v>
       </c>
       <c r="H171" t="str">
         <v/>
       </c>
       <c r="I171" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="172">
@@ -5378,13 +5378,13 @@
         <v>Passed</v>
       </c>
       <c r="G172" t="str">
-        <v>405ms</v>
+        <v>542ms</v>
       </c>
       <c r="H172" t="str">
         <v/>
       </c>
       <c r="I172" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="173">
@@ -5407,13 +5407,13 @@
         <v>Passed</v>
       </c>
       <c r="G173" t="str">
-        <v>174ms</v>
+        <v>127ms</v>
       </c>
       <c r="H173" t="str">
         <v/>
       </c>
       <c r="I173" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="174">
@@ -5436,13 +5436,13 @@
         <v>Passed</v>
       </c>
       <c r="G174" t="str">
-        <v>115ms</v>
+        <v>164ms</v>
       </c>
       <c r="H174" t="str">
         <v/>
       </c>
       <c r="I174" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="175">
@@ -5465,13 +5465,13 @@
         <v>Passed</v>
       </c>
       <c r="G175" t="str">
-        <v>147ms</v>
+        <v>149ms</v>
       </c>
       <c r="H175" t="str">
         <v/>
       </c>
       <c r="I175" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="176">
@@ -5494,13 +5494,13 @@
         <v>Passed</v>
       </c>
       <c r="G176" t="str">
-        <v>152ms</v>
+        <v>456ms</v>
       </c>
       <c r="H176" t="str">
         <v/>
       </c>
       <c r="I176" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="177">
@@ -5523,13 +5523,13 @@
         <v>Passed</v>
       </c>
       <c r="G177" t="str">
-        <v>451ms</v>
+        <v>455ms</v>
       </c>
       <c r="H177" t="str">
         <v/>
       </c>
       <c r="I177" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="178">
@@ -5552,13 +5552,13 @@
         <v>Passed</v>
       </c>
       <c r="G178" t="str">
-        <v>469ms</v>
+        <v>359ms</v>
       </c>
       <c r="H178" t="str">
         <v/>
       </c>
       <c r="I178" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="179">
@@ -5581,13 +5581,13 @@
         <v>Passed</v>
       </c>
       <c r="G179" t="str">
-        <v>543ms</v>
+        <v>546ms</v>
       </c>
       <c r="H179" t="str">
         <v/>
       </c>
       <c r="I179" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.487Z</v>
       </c>
     </row>
     <row r="180">
@@ -5610,13 +5610,13 @@
         <v>Passed</v>
       </c>
       <c r="G180" t="str">
-        <v>526ms</v>
+        <v>595ms</v>
       </c>
       <c r="H180" t="str">
         <v/>
       </c>
       <c r="I180" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="181">
@@ -5639,13 +5639,13 @@
         <v>Passed</v>
       </c>
       <c r="G181" t="str">
-        <v>319ms</v>
+        <v>305ms</v>
       </c>
       <c r="H181" t="str">
         <v/>
       </c>
       <c r="I181" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="182">
@@ -5668,13 +5668,13 @@
         <v>Passed</v>
       </c>
       <c r="G182" t="str">
-        <v>181ms</v>
+        <v>221ms</v>
       </c>
       <c r="H182" t="str">
         <v/>
       </c>
       <c r="I182" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="183">
@@ -5697,13 +5697,13 @@
         <v>Passed</v>
       </c>
       <c r="G183" t="str">
-        <v>533ms</v>
+        <v>329ms</v>
       </c>
       <c r="H183" t="str">
         <v/>
       </c>
       <c r="I183" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="184">
@@ -5726,13 +5726,13 @@
         <v>Passed</v>
       </c>
       <c r="G184" t="str">
-        <v>441ms</v>
+        <v>402ms</v>
       </c>
       <c r="H184" t="str">
         <v/>
       </c>
       <c r="I184" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="185">
@@ -5755,13 +5755,13 @@
         <v>Passed</v>
       </c>
       <c r="G185" t="str">
-        <v>558ms</v>
+        <v>122ms</v>
       </c>
       <c r="H185" t="str">
         <v/>
       </c>
       <c r="I185" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="186">
@@ -5784,13 +5784,13 @@
         <v>Passed</v>
       </c>
       <c r="G186" t="str">
-        <v>219ms</v>
+        <v>140ms</v>
       </c>
       <c r="H186" t="str">
         <v/>
       </c>
       <c r="I186" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="187">
@@ -5813,13 +5813,13 @@
         <v>Passed</v>
       </c>
       <c r="G187" t="str">
-        <v>161ms</v>
+        <v>578ms</v>
       </c>
       <c r="H187" t="str">
         <v/>
       </c>
       <c r="I187" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="188">
@@ -5842,13 +5842,13 @@
         <v>Passed</v>
       </c>
       <c r="G188" t="str">
-        <v>370ms</v>
+        <v>278ms</v>
       </c>
       <c r="H188" t="str">
         <v/>
       </c>
       <c r="I188" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="189">
@@ -5871,13 +5871,13 @@
         <v>Skipped</v>
       </c>
       <c r="G189" t="str">
-        <v>168ms</v>
+        <v>577ms</v>
       </c>
       <c r="H189" t="str">
         <v/>
       </c>
       <c r="I189" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="190">
@@ -5900,13 +5900,13 @@
         <v>Passed</v>
       </c>
       <c r="G190" t="str">
-        <v>245ms</v>
+        <v>391ms</v>
       </c>
       <c r="H190" t="str">
         <v/>
       </c>
       <c r="I190" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="191">
@@ -5929,13 +5929,13 @@
         <v>Passed</v>
       </c>
       <c r="G191" t="str">
-        <v>334ms</v>
+        <v>192ms</v>
       </c>
       <c r="H191" t="str">
         <v/>
       </c>
       <c r="I191" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="192">
@@ -5958,13 +5958,13 @@
         <v>Passed</v>
       </c>
       <c r="G192" t="str">
-        <v>521ms</v>
+        <v>265ms</v>
       </c>
       <c r="H192" t="str">
         <v/>
       </c>
       <c r="I192" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="193">
@@ -5987,13 +5987,13 @@
         <v>Passed</v>
       </c>
       <c r="G193" t="str">
-        <v>217ms</v>
+        <v>275ms</v>
       </c>
       <c r="H193" t="str">
         <v/>
       </c>
       <c r="I193" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="194">
@@ -6016,13 +6016,13 @@
         <v>Passed</v>
       </c>
       <c r="G194" t="str">
-        <v>303ms</v>
+        <v>259ms</v>
       </c>
       <c r="H194" t="str">
         <v/>
       </c>
       <c r="I194" t="str">
-        <v>2026-08-26T06:43:35.413Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="195">
@@ -6045,13 +6045,13 @@
         <v>Passed</v>
       </c>
       <c r="G195" t="str">
-        <v>545ms</v>
+        <v>586ms</v>
       </c>
       <c r="H195" t="str">
         <v/>
       </c>
       <c r="I195" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="196">
@@ -6074,13 +6074,13 @@
         <v>Passed</v>
       </c>
       <c r="G196" t="str">
-        <v>520ms</v>
+        <v>392ms</v>
       </c>
       <c r="H196" t="str">
         <v/>
       </c>
       <c r="I196" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="197">
@@ -6103,13 +6103,13 @@
         <v>Passed</v>
       </c>
       <c r="G197" t="str">
-        <v>464ms</v>
+        <v>335ms</v>
       </c>
       <c r="H197" t="str">
         <v/>
       </c>
       <c r="I197" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="198">
@@ -6132,13 +6132,13 @@
         <v>Passed</v>
       </c>
       <c r="G198" t="str">
-        <v>218ms</v>
+        <v>169ms</v>
       </c>
       <c r="H198" t="str">
         <v/>
       </c>
       <c r="I198" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="199">
@@ -6161,13 +6161,13 @@
         <v>Passed</v>
       </c>
       <c r="G199" t="str">
-        <v>279ms</v>
+        <v>290ms</v>
       </c>
       <c r="H199" t="str">
         <v/>
       </c>
       <c r="I199" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="200">
@@ -6190,13 +6190,13 @@
         <v>Passed</v>
       </c>
       <c r="G200" t="str">
-        <v>351ms</v>
+        <v>578ms</v>
       </c>
       <c r="H200" t="str">
         <v/>
       </c>
       <c r="I200" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="201">
@@ -6219,13 +6219,13 @@
         <v>Passed</v>
       </c>
       <c r="G201" t="str">
-        <v>278ms</v>
+        <v>238ms</v>
       </c>
       <c r="H201" t="str">
         <v/>
       </c>
       <c r="I201" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="202">
@@ -6248,13 +6248,13 @@
         <v>Passed</v>
       </c>
       <c r="G202" t="str">
-        <v>470ms</v>
+        <v>438ms</v>
       </c>
       <c r="H202" t="str">
         <v/>
       </c>
       <c r="I202" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.488Z</v>
       </c>
     </row>
     <row r="203">
@@ -6277,13 +6277,13 @@
         <v>Passed</v>
       </c>
       <c r="G203" t="str">
-        <v>121ms</v>
+        <v>556ms</v>
       </c>
       <c r="H203" t="str">
         <v/>
       </c>
       <c r="I203" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="204">
@@ -6306,13 +6306,13 @@
         <v>Passed</v>
       </c>
       <c r="G204" t="str">
-        <v>330ms</v>
+        <v>277ms</v>
       </c>
       <c r="H204" t="str">
         <v/>
       </c>
       <c r="I204" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="205">
@@ -6335,13 +6335,13 @@
         <v>Passed</v>
       </c>
       <c r="G205" t="str">
-        <v>409ms</v>
+        <v>350ms</v>
       </c>
       <c r="H205" t="str">
         <v/>
       </c>
       <c r="I205" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="206">
@@ -6364,13 +6364,13 @@
         <v>Passed</v>
       </c>
       <c r="G206" t="str">
-        <v>315ms</v>
+        <v>458ms</v>
       </c>
       <c r="H206" t="str">
         <v/>
       </c>
       <c r="I206" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="207">
@@ -6393,13 +6393,13 @@
         <v>Passed</v>
       </c>
       <c r="G207" t="str">
-        <v>546ms</v>
+        <v>342ms</v>
       </c>
       <c r="H207" t="str">
         <v/>
       </c>
       <c r="I207" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="208">
@@ -6422,13 +6422,13 @@
         <v>Passed</v>
       </c>
       <c r="G208" t="str">
-        <v>306ms</v>
+        <v>547ms</v>
       </c>
       <c r="H208" t="str">
         <v/>
       </c>
       <c r="I208" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="209">
@@ -6451,13 +6451,13 @@
         <v>Passed</v>
       </c>
       <c r="G209" t="str">
-        <v>207ms</v>
+        <v>293ms</v>
       </c>
       <c r="H209" t="str">
         <v/>
       </c>
       <c r="I209" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="210">
@@ -6480,13 +6480,13 @@
         <v>Passed</v>
       </c>
       <c r="G210" t="str">
-        <v>536ms</v>
+        <v>106ms</v>
       </c>
       <c r="H210" t="str">
         <v/>
       </c>
       <c r="I210" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="211">
@@ -6509,13 +6509,13 @@
         <v>Passed</v>
       </c>
       <c r="G211" t="str">
-        <v>104ms</v>
+        <v>169ms</v>
       </c>
       <c r="H211" t="str">
         <v/>
       </c>
       <c r="I211" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="212">
@@ -6538,13 +6538,13 @@
         <v>Passed</v>
       </c>
       <c r="G212" t="str">
-        <v>494ms</v>
+        <v>341ms</v>
       </c>
       <c r="H212" t="str">
         <v/>
       </c>
       <c r="I212" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="213">
@@ -6567,13 +6567,13 @@
         <v>Passed</v>
       </c>
       <c r="G213" t="str">
-        <v>535ms</v>
+        <v>424ms</v>
       </c>
       <c r="H213" t="str">
         <v/>
       </c>
       <c r="I213" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="214">
@@ -6596,13 +6596,13 @@
         <v>Passed</v>
       </c>
       <c r="G214" t="str">
-        <v>371ms</v>
+        <v>517ms</v>
       </c>
       <c r="H214" t="str">
         <v/>
       </c>
       <c r="I214" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="215">
@@ -6625,13 +6625,13 @@
         <v>Passed</v>
       </c>
       <c r="G215" t="str">
-        <v>143ms</v>
+        <v>491ms</v>
       </c>
       <c r="H215" t="str">
         <v/>
       </c>
       <c r="I215" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="216">
@@ -6654,13 +6654,13 @@
         <v>Passed</v>
       </c>
       <c r="G216" t="str">
-        <v>416ms</v>
+        <v>350ms</v>
       </c>
       <c r="H216" t="str">
         <v/>
       </c>
       <c r="I216" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="217">
@@ -6683,13 +6683,13 @@
         <v>Passed</v>
       </c>
       <c r="G217" t="str">
-        <v>422ms</v>
+        <v>194ms</v>
       </c>
       <c r="H217" t="str">
         <v/>
       </c>
       <c r="I217" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="218">
@@ -6712,13 +6712,13 @@
         <v>Passed</v>
       </c>
       <c r="G218" t="str">
-        <v>549ms</v>
+        <v>248ms</v>
       </c>
       <c r="H218" t="str">
         <v/>
       </c>
       <c r="I218" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="219">
@@ -6741,13 +6741,13 @@
         <v>Skipped</v>
       </c>
       <c r="G219" t="str">
-        <v>296ms</v>
+        <v>564ms</v>
       </c>
       <c r="H219" t="str">
         <v/>
       </c>
       <c r="I219" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="220">
@@ -6770,13 +6770,13 @@
         <v>Passed</v>
       </c>
       <c r="G220" t="str">
-        <v>372ms</v>
+        <v>328ms</v>
       </c>
       <c r="H220" t="str">
         <v/>
       </c>
       <c r="I220" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="221">
@@ -6799,13 +6799,13 @@
         <v>Passed</v>
       </c>
       <c r="G221" t="str">
-        <v>341ms</v>
+        <v>422ms</v>
       </c>
       <c r="H221" t="str">
         <v/>
       </c>
       <c r="I221" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="222">
@@ -6828,13 +6828,13 @@
         <v>Passed</v>
       </c>
       <c r="G222" t="str">
-        <v>417ms</v>
+        <v>375ms</v>
       </c>
       <c r="H222" t="str">
         <v/>
       </c>
       <c r="I222" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="223">
@@ -6857,13 +6857,13 @@
         <v>Passed</v>
       </c>
       <c r="G223" t="str">
-        <v>232ms</v>
+        <v>134ms</v>
       </c>
       <c r="H223" t="str">
         <v/>
       </c>
       <c r="I223" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="224">
@@ -6886,13 +6886,13 @@
         <v>Passed</v>
       </c>
       <c r="G224" t="str">
-        <v>573ms</v>
+        <v>225ms</v>
       </c>
       <c r="H224" t="str">
         <v/>
       </c>
       <c r="I224" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="225">
@@ -6915,13 +6915,13 @@
         <v>Passed</v>
       </c>
       <c r="G225" t="str">
-        <v>198ms</v>
+        <v>250ms</v>
       </c>
       <c r="H225" t="str">
         <v/>
       </c>
       <c r="I225" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="226">
@@ -6944,13 +6944,13 @@
         <v>Passed</v>
       </c>
       <c r="G226" t="str">
-        <v>207ms</v>
+        <v>228ms</v>
       </c>
       <c r="H226" t="str">
         <v/>
       </c>
       <c r="I226" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="227">
@@ -6973,13 +6973,13 @@
         <v>Passed</v>
       </c>
       <c r="G227" t="str">
-        <v>363ms</v>
+        <v>338ms</v>
       </c>
       <c r="H227" t="str">
         <v/>
       </c>
       <c r="I227" t="str">
-        <v>2026-08-26T06:43:35.414Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="228">
@@ -7002,13 +7002,13 @@
         <v>Passed</v>
       </c>
       <c r="G228" t="str">
-        <v>133ms</v>
+        <v>290ms</v>
       </c>
       <c r="H228" t="str">
         <v/>
       </c>
       <c r="I228" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="229">
@@ -7031,13 +7031,13 @@
         <v>Passed</v>
       </c>
       <c r="G229" t="str">
-        <v>214ms</v>
+        <v>282ms</v>
       </c>
       <c r="H229" t="str">
         <v/>
       </c>
       <c r="I229" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="230">
@@ -7060,13 +7060,13 @@
         <v>Passed</v>
       </c>
       <c r="G230" t="str">
-        <v>233ms</v>
+        <v>130ms</v>
       </c>
       <c r="H230" t="str">
         <v/>
       </c>
       <c r="I230" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="231">
@@ -7089,13 +7089,13 @@
         <v>Passed</v>
       </c>
       <c r="G231" t="str">
-        <v>362ms</v>
+        <v>465ms</v>
       </c>
       <c r="H231" t="str">
         <v/>
       </c>
       <c r="I231" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.489Z</v>
       </c>
     </row>
     <row r="232">
@@ -7118,13 +7118,13 @@
         <v>Passed</v>
       </c>
       <c r="G232" t="str">
-        <v>513ms</v>
+        <v>273ms</v>
       </c>
       <c r="H232" t="str">
         <v/>
       </c>
       <c r="I232" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="233">
@@ -7147,13 +7147,13 @@
         <v>Passed</v>
       </c>
       <c r="G233" t="str">
-        <v>235ms</v>
+        <v>242ms</v>
       </c>
       <c r="H233" t="str">
         <v/>
       </c>
       <c r="I233" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="234">
@@ -7176,13 +7176,13 @@
         <v>Passed</v>
       </c>
       <c r="G234" t="str">
-        <v>571ms</v>
+        <v>268ms</v>
       </c>
       <c r="H234" t="str">
         <v/>
       </c>
       <c r="I234" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="235">
@@ -7205,13 +7205,13 @@
         <v>Passed</v>
       </c>
       <c r="G235" t="str">
-        <v>352ms</v>
+        <v>321ms</v>
       </c>
       <c r="H235" t="str">
         <v/>
       </c>
       <c r="I235" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="236">
@@ -7234,13 +7234,13 @@
         <v>Passed</v>
       </c>
       <c r="G236" t="str">
-        <v>179ms</v>
+        <v>507ms</v>
       </c>
       <c r="H236" t="str">
         <v/>
       </c>
       <c r="I236" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="237">
@@ -7263,13 +7263,13 @@
         <v>Passed</v>
       </c>
       <c r="G237" t="str">
-        <v>221ms</v>
+        <v>347ms</v>
       </c>
       <c r="H237" t="str">
         <v/>
       </c>
       <c r="I237" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="238">
@@ -7292,13 +7292,13 @@
         <v>Passed</v>
       </c>
       <c r="G238" t="str">
-        <v>231ms</v>
+        <v>530ms</v>
       </c>
       <c r="H238" t="str">
         <v/>
       </c>
       <c r="I238" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="239">
@@ -7321,13 +7321,13 @@
         <v>Passed</v>
       </c>
       <c r="G239" t="str">
-        <v>423ms</v>
+        <v>382ms</v>
       </c>
       <c r="H239" t="str">
         <v/>
       </c>
       <c r="I239" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="240">
@@ -7350,13 +7350,13 @@
         <v>Passed</v>
       </c>
       <c r="G240" t="str">
-        <v>363ms</v>
+        <v>348ms</v>
       </c>
       <c r="H240" t="str">
         <v/>
       </c>
       <c r="I240" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="241">
@@ -7379,13 +7379,13 @@
         <v>Passed</v>
       </c>
       <c r="G241" t="str">
-        <v>377ms</v>
+        <v>107ms</v>
       </c>
       <c r="H241" t="str">
         <v/>
       </c>
       <c r="I241" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="242">
@@ -7408,13 +7408,13 @@
         <v>Passed</v>
       </c>
       <c r="G242" t="str">
-        <v>296ms</v>
+        <v>158ms</v>
       </c>
       <c r="H242" t="str">
         <v/>
       </c>
       <c r="I242" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="243">
@@ -7437,13 +7437,13 @@
         <v>Passed</v>
       </c>
       <c r="G243" t="str">
-        <v>422ms</v>
+        <v>106ms</v>
       </c>
       <c r="H243" t="str">
         <v/>
       </c>
       <c r="I243" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="244">
@@ -7466,13 +7466,13 @@
         <v>Passed</v>
       </c>
       <c r="G244" t="str">
-        <v>194ms</v>
+        <v>596ms</v>
       </c>
       <c r="H244" t="str">
         <v/>
       </c>
       <c r="I244" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="245">
@@ -7495,13 +7495,13 @@
         <v>Passed</v>
       </c>
       <c r="G245" t="str">
-        <v>435ms</v>
+        <v>418ms</v>
       </c>
       <c r="H245" t="str">
         <v/>
       </c>
       <c r="I245" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="246">
@@ -7524,13 +7524,13 @@
         <v>Passed</v>
       </c>
       <c r="G246" t="str">
-        <v>493ms</v>
+        <v>428ms</v>
       </c>
       <c r="H246" t="str">
         <v/>
       </c>
       <c r="I246" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="247">
@@ -7553,13 +7553,13 @@
         <v>Passed</v>
       </c>
       <c r="G247" t="str">
-        <v>590ms</v>
+        <v>411ms</v>
       </c>
       <c r="H247" t="str">
         <v/>
       </c>
       <c r="I247" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="248">
@@ -7582,13 +7582,13 @@
         <v>Passed</v>
       </c>
       <c r="G248" t="str">
-        <v>459ms</v>
+        <v>271ms</v>
       </c>
       <c r="H248" t="str">
         <v/>
       </c>
       <c r="I248" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="249">
@@ -7611,13 +7611,13 @@
         <v>Skipped</v>
       </c>
       <c r="G249" t="str">
-        <v>109ms</v>
+        <v>203ms</v>
       </c>
       <c r="H249" t="str">
         <v/>
       </c>
       <c r="I249" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.490Z</v>
       </c>
     </row>
     <row r="250">
@@ -7640,13 +7640,13 @@
         <v>Passed</v>
       </c>
       <c r="G250" t="str">
-        <v>417ms</v>
+        <v>214ms</v>
       </c>
       <c r="H250" t="str">
         <v/>
       </c>
       <c r="I250" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="251">
@@ -7669,13 +7669,13 @@
         <v>Passed</v>
       </c>
       <c r="G251" t="str">
-        <v>508ms</v>
+        <v>418ms</v>
       </c>
       <c r="H251" t="str">
         <v/>
       </c>
       <c r="I251" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="252">
@@ -7698,13 +7698,13 @@
         <v>Passed</v>
       </c>
       <c r="G252" t="str">
-        <v>517ms</v>
+        <v>597ms</v>
       </c>
       <c r="H252" t="str">
         <v/>
       </c>
       <c r="I252" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="253">
@@ -7727,13 +7727,13 @@
         <v>Passed</v>
       </c>
       <c r="G253" t="str">
-        <v>192ms</v>
+        <v>360ms</v>
       </c>
       <c r="H253" t="str">
         <v/>
       </c>
       <c r="I253" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="254">
@@ -7756,13 +7756,13 @@
         <v>Passed</v>
       </c>
       <c r="G254" t="str">
-        <v>167ms</v>
+        <v>122ms</v>
       </c>
       <c r="H254" t="str">
         <v/>
       </c>
       <c r="I254" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="255">
@@ -7785,13 +7785,13 @@
         <v>Passed</v>
       </c>
       <c r="G255" t="str">
-        <v>162ms</v>
+        <v>349ms</v>
       </c>
       <c r="H255" t="str">
         <v/>
       </c>
       <c r="I255" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="256">
@@ -7814,13 +7814,13 @@
         <v>Passed</v>
       </c>
       <c r="G256" t="str">
-        <v>590ms</v>
+        <v>457ms</v>
       </c>
       <c r="H256" t="str">
         <v/>
       </c>
       <c r="I256" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="257">
@@ -7843,13 +7843,13 @@
         <v>Passed</v>
       </c>
       <c r="G257" t="str">
-        <v>294ms</v>
+        <v>542ms</v>
       </c>
       <c r="H257" t="str">
         <v/>
       </c>
       <c r="I257" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="258">
@@ -7872,13 +7872,13 @@
         <v>Passed</v>
       </c>
       <c r="G258" t="str">
-        <v>130ms</v>
+        <v>287ms</v>
       </c>
       <c r="H258" t="str">
         <v/>
       </c>
       <c r="I258" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="259">
@@ -7901,13 +7901,13 @@
         <v>Passed</v>
       </c>
       <c r="G259" t="str">
-        <v>503ms</v>
+        <v>301ms</v>
       </c>
       <c r="H259" t="str">
         <v/>
       </c>
       <c r="I259" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="260">
@@ -7930,13 +7930,13 @@
         <v>Passed</v>
       </c>
       <c r="G260" t="str">
-        <v>498ms</v>
+        <v>354ms</v>
       </c>
       <c r="H260" t="str">
         <v/>
       </c>
       <c r="I260" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="261">
@@ -7959,13 +7959,13 @@
         <v>Passed</v>
       </c>
       <c r="G261" t="str">
-        <v>533ms</v>
+        <v>369ms</v>
       </c>
       <c r="H261" t="str">
         <v/>
       </c>
       <c r="I261" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="262">
@@ -7988,13 +7988,13 @@
         <v>Passed</v>
       </c>
       <c r="G262" t="str">
-        <v>208ms</v>
+        <v>114ms</v>
       </c>
       <c r="H262" t="str">
         <v/>
       </c>
       <c r="I262" t="str">
-        <v>2026-08-26T06:43:35.415Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="263">
@@ -8017,13 +8017,13 @@
         <v>Passed</v>
       </c>
       <c r="G263" t="str">
-        <v>409ms</v>
+        <v>293ms</v>
       </c>
       <c r="H263" t="str">
         <v/>
       </c>
       <c r="I263" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="264">
@@ -8046,13 +8046,13 @@
         <v>Passed</v>
       </c>
       <c r="G264" t="str">
-        <v>297ms</v>
+        <v>318ms</v>
       </c>
       <c r="H264" t="str">
         <v/>
       </c>
       <c r="I264" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="265">
@@ -8075,13 +8075,13 @@
         <v>Passed</v>
       </c>
       <c r="G265" t="str">
-        <v>206ms</v>
+        <v>499ms</v>
       </c>
       <c r="H265" t="str">
         <v/>
       </c>
       <c r="I265" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="266">
@@ -8104,13 +8104,13 @@
         <v>Passed</v>
       </c>
       <c r="G266" t="str">
-        <v>488ms</v>
+        <v>278ms</v>
       </c>
       <c r="H266" t="str">
         <v/>
       </c>
       <c r="I266" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="267">
@@ -8133,13 +8133,13 @@
         <v>Passed</v>
       </c>
       <c r="G267" t="str">
-        <v>143ms</v>
+        <v>413ms</v>
       </c>
       <c r="H267" t="str">
         <v/>
       </c>
       <c r="I267" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="268">
@@ -8162,13 +8162,13 @@
         <v>Passed</v>
       </c>
       <c r="G268" t="str">
-        <v>252ms</v>
+        <v>449ms</v>
       </c>
       <c r="H268" t="str">
         <v/>
       </c>
       <c r="I268" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="269">
@@ -8191,13 +8191,13 @@
         <v>Passed</v>
       </c>
       <c r="G269" t="str">
-        <v>163ms</v>
+        <v>396ms</v>
       </c>
       <c r="H269" t="str">
         <v/>
       </c>
       <c r="I269" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="270">
@@ -8220,13 +8220,13 @@
         <v>Passed</v>
       </c>
       <c r="G270" t="str">
-        <v>516ms</v>
+        <v>566ms</v>
       </c>
       <c r="H270" t="str">
         <v/>
       </c>
       <c r="I270" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="271">
@@ -8249,13 +8249,13 @@
         <v>Passed</v>
       </c>
       <c r="G271" t="str">
-        <v>545ms</v>
+        <v>573ms</v>
       </c>
       <c r="H271" t="str">
         <v/>
       </c>
       <c r="I271" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="272">
@@ -8278,13 +8278,13 @@
         <v>Passed</v>
       </c>
       <c r="G272" t="str">
-        <v>102ms</v>
+        <v>234ms</v>
       </c>
       <c r="H272" t="str">
         <v/>
       </c>
       <c r="I272" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="273">
@@ -8307,13 +8307,13 @@
         <v>Passed</v>
       </c>
       <c r="G273" t="str">
-        <v>544ms</v>
+        <v>269ms</v>
       </c>
       <c r="H273" t="str">
         <v/>
       </c>
       <c r="I273" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="274">
@@ -8336,13 +8336,13 @@
         <v>Passed</v>
       </c>
       <c r="G274" t="str">
-        <v>334ms</v>
+        <v>571ms</v>
       </c>
       <c r="H274" t="str">
         <v/>
       </c>
       <c r="I274" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="275">
@@ -8365,13 +8365,13 @@
         <v>Passed</v>
       </c>
       <c r="G275" t="str">
-        <v>294ms</v>
+        <v>357ms</v>
       </c>
       <c r="H275" t="str">
         <v/>
       </c>
       <c r="I275" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="276">
@@ -8394,13 +8394,13 @@
         <v>Passed</v>
       </c>
       <c r="G276" t="str">
-        <v>254ms</v>
+        <v>134ms</v>
       </c>
       <c r="H276" t="str">
         <v/>
       </c>
       <c r="I276" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="277">
@@ -8423,13 +8423,13 @@
         <v>Passed</v>
       </c>
       <c r="G277" t="str">
-        <v>517ms</v>
+        <v>433ms</v>
       </c>
       <c r="H277" t="str">
         <v/>
       </c>
       <c r="I277" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="278">
@@ -8452,13 +8452,13 @@
         <v>Passed</v>
       </c>
       <c r="G278" t="str">
-        <v>513ms</v>
+        <v>489ms</v>
       </c>
       <c r="H278" t="str">
         <v/>
       </c>
       <c r="I278" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="279">
@@ -8481,13 +8481,13 @@
         <v>Passed</v>
       </c>
       <c r="G279" t="str">
-        <v>224ms</v>
+        <v>314ms</v>
       </c>
       <c r="H279" t="str">
         <v/>
       </c>
       <c r="I279" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="280">
@@ -8510,13 +8510,13 @@
         <v>Passed</v>
       </c>
       <c r="G280" t="str">
-        <v>217ms</v>
+        <v>132ms</v>
       </c>
       <c r="H280" t="str">
         <v/>
       </c>
       <c r="I280" t="str">
-        <v>2026-08-26T06:43:35.416Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="281">
@@ -8539,13 +8539,13 @@
         <v>Passed</v>
       </c>
       <c r="G281" t="str">
-        <v>233ms</v>
+        <v>560ms</v>
       </c>
       <c r="H281" t="str">
         <v/>
       </c>
       <c r="I281" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="282">
@@ -8568,13 +8568,13 @@
         <v>Passed</v>
       </c>
       <c r="G282" t="str">
-        <v>348ms</v>
+        <v>503ms</v>
       </c>
       <c r="H282" t="str">
         <v/>
       </c>
       <c r="I282" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="283">
@@ -8597,13 +8597,13 @@
         <v>Passed</v>
       </c>
       <c r="G283" t="str">
-        <v>338ms</v>
+        <v>341ms</v>
       </c>
       <c r="H283" t="str">
         <v/>
       </c>
       <c r="I283" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.491Z</v>
       </c>
     </row>
     <row r="284">
@@ -8626,13 +8626,13 @@
         <v>Passed</v>
       </c>
       <c r="G284" t="str">
-        <v>396ms</v>
+        <v>188ms</v>
       </c>
       <c r="H284" t="str">
         <v/>
       </c>
       <c r="I284" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.492Z</v>
       </c>
     </row>
     <row r="285">
@@ -8655,13 +8655,13 @@
         <v>Passed</v>
       </c>
       <c r="G285" t="str">
-        <v>234ms</v>
+        <v>228ms</v>
       </c>
       <c r="H285" t="str">
         <v/>
       </c>
       <c r="I285" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="286">
@@ -8684,13 +8684,13 @@
         <v>Passed</v>
       </c>
       <c r="G286" t="str">
-        <v>255ms</v>
+        <v>375ms</v>
       </c>
       <c r="H286" t="str">
         <v/>
       </c>
       <c r="I286" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="287">
@@ -8713,13 +8713,13 @@
         <v>Passed</v>
       </c>
       <c r="G287" t="str">
-        <v>577ms</v>
+        <v>356ms</v>
       </c>
       <c r="H287" t="str">
         <v/>
       </c>
       <c r="I287" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="288">
@@ -8742,13 +8742,13 @@
         <v>Passed</v>
       </c>
       <c r="G288" t="str">
-        <v>297ms</v>
+        <v>498ms</v>
       </c>
       <c r="H288" t="str">
         <v/>
       </c>
       <c r="I288" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="289">
@@ -8771,13 +8771,13 @@
         <v>Passed</v>
       </c>
       <c r="G289" t="str">
-        <v>170ms</v>
+        <v>400ms</v>
       </c>
       <c r="H289" t="str">
         <v/>
       </c>
       <c r="I289" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="290">
@@ -8800,13 +8800,13 @@
         <v>Passed</v>
       </c>
       <c r="G290" t="str">
-        <v>292ms</v>
+        <v>443ms</v>
       </c>
       <c r="H290" t="str">
         <v/>
       </c>
       <c r="I290" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="291">
@@ -8829,13 +8829,13 @@
         <v>Passed</v>
       </c>
       <c r="G291" t="str">
-        <v>117ms</v>
+        <v>262ms</v>
       </c>
       <c r="H291" t="str">
         <v/>
       </c>
       <c r="I291" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="292">
@@ -8858,13 +8858,13 @@
         <v>Passed</v>
       </c>
       <c r="G292" t="str">
-        <v>533ms</v>
+        <v>527ms</v>
       </c>
       <c r="H292" t="str">
         <v/>
       </c>
       <c r="I292" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="293">
@@ -8887,13 +8887,13 @@
         <v>Passed</v>
       </c>
       <c r="G293" t="str">
-        <v>310ms</v>
+        <v>128ms</v>
       </c>
       <c r="H293" t="str">
         <v/>
       </c>
       <c r="I293" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="294">
@@ -8916,13 +8916,13 @@
         <v>Passed</v>
       </c>
       <c r="G294" t="str">
-        <v>400ms</v>
+        <v>232ms</v>
       </c>
       <c r="H294" t="str">
         <v/>
       </c>
       <c r="I294" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="295">
@@ -8945,13 +8945,13 @@
         <v>Passed</v>
       </c>
       <c r="G295" t="str">
-        <v>458ms</v>
+        <v>211ms</v>
       </c>
       <c r="H295" t="str">
         <v/>
       </c>
       <c r="I295" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="296">
@@ -8974,13 +8974,13 @@
         <v>Passed</v>
       </c>
       <c r="G296" t="str">
-        <v>294ms</v>
+        <v>122ms</v>
       </c>
       <c r="H296" t="str">
         <v/>
       </c>
       <c r="I296" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="297">
@@ -9003,13 +9003,13 @@
         <v>Passed</v>
       </c>
       <c r="G297" t="str">
-        <v>176ms</v>
+        <v>417ms</v>
       </c>
       <c r="H297" t="str">
         <v/>
       </c>
       <c r="I297" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="298">
@@ -9032,13 +9032,13 @@
         <v>Passed</v>
       </c>
       <c r="G298" t="str">
-        <v>318ms</v>
+        <v>301ms</v>
       </c>
       <c r="H298" t="str">
         <v/>
       </c>
       <c r="I298" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="299">
@@ -9061,13 +9061,13 @@
         <v>Passed</v>
       </c>
       <c r="G299" t="str">
-        <v>528ms</v>
+        <v>361ms</v>
       </c>
       <c r="H299" t="str">
         <v/>
       </c>
       <c r="I299" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="300">
@@ -9090,13 +9090,13 @@
         <v>Passed</v>
       </c>
       <c r="G300" t="str">
-        <v>218ms</v>
+        <v>184ms</v>
       </c>
       <c r="H300" t="str">
         <v/>
       </c>
       <c r="I300" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
     <row r="301">
@@ -9119,13 +9119,13 @@
         <v>Passed</v>
       </c>
       <c r="G301" t="str">
-        <v>166ms</v>
+        <v>486ms</v>
       </c>
       <c r="H301" t="str">
         <v/>
       </c>
       <c r="I301" t="str">
-        <v>2026-08-26T06:43:35.417Z</v>
+        <v>2026-09-08T05:53:03.493Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>